<commit_message>
this simpler version has upload counts hide counts and miscoutn models as well as search models
</commit_message>
<xml_diff>
--- a/public/samples/lg-200-model-counts.xlsx
+++ b/public/samples/lg-200-model-counts.xlsx
@@ -1926,10 +1926,10 @@
         <v>Yes</v>
       </c>
       <c r="E76">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F76">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="77">
@@ -1937,7 +1937,7 @@
         <v>B006</v>
       </c>
       <c r="B77" t="str">
-        <v>WM3700HWA</v>
+        <v>LCFS22EXS</v>
       </c>
       <c r="C77" t="str">
         <v>Completed</v>
@@ -1949,7 +1949,7 @@
         <v>10</v>
       </c>
       <c r="F77">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="78">
@@ -1983,13 +1983,13 @@
         <v>Completed</v>
       </c>
       <c r="D79" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="E79">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F79">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="80">
@@ -4340,16 +4340,16 @@
         <v>LRFVS3006D</v>
       </c>
       <c r="C197" t="str">
-        <v>Not Started</v>
+        <v>Completed</v>
       </c>
       <c r="D197" t="str">
-        <v/>
+        <v>Yes</v>
       </c>
       <c r="E197">
         <v>10</v>
       </c>
-      <c r="F197" t="str">
-        <v/>
+      <c r="F197">
+        <v>13</v>
       </c>
     </row>
     <row r="198">
@@ -4917,19 +4917,19 @@
         <v>D050</v>
       </c>
       <c r="B226" t="str">
-        <v>DLGX5681V</v>
+        <v>LRFVS3006D</v>
       </c>
       <c r="C226" t="str">
         <v>Completed</v>
       </c>
       <c r="D226" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="E226">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F226">
-        <v>17</v>
+        <v>7</v>
       </c>
     </row>
     <row r="227">
@@ -14297,19 +14297,19 @@
         <v>M055</v>
       </c>
       <c r="B695" t="str">
-        <v>LDT5678ST</v>
+        <v>LFXS29626W</v>
       </c>
       <c r="C695" t="str">
         <v>Completed</v>
       </c>
       <c r="D695" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="E695">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F695">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="696">
@@ -33142,7 +33142,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <cols>
     <col min="1" max="1" width="44.83203125" customWidth="1"/>
     <col min="2" max="2" width="115.83203125" customWidth="1"/>
@@ -33174,7 +33174,7 @@
         <v>Matching counted bays (green)</v>
       </c>
       <c r="B4">
-        <v>1464</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="5">
@@ -33182,7 +33182,7 @@
         <v>Discrepant counted bays (red)</v>
       </c>
       <c r="B5">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
@@ -33198,7 +33198,7 @@
         <v>Not counted (blank Count Qty A-B)</v>
       </c>
       <c r="B7">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8">
@@ -33238,60 +33238,68 @@
         <v>Scope</v>
       </c>
       <c r="B12" t="str">
-        <v>The current uploader updates count colors only. Inventory model lists and orders still come from the inventory feed.</v>
+        <v>Uploads provide count colors, miscount totals, and offset arrows. Inventory model labels and orders still use the feed.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Not Started</v>
+        <v>Offset pairs</v>
       </c>
       <c r="B13" t="str">
-        <v>Leave Count Qty A-B blank; zero is a recorded count of zero.</v>
+        <v>B005 to B006: 4 units vertically; D010 to D050: 3 units horizontally; B008 to M055: 5 units across the warehouse. Arrows indicate possible offsets, not confirmed transfers.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Models</v>
+        <v>Not Started</v>
       </c>
       <c r="B14" t="str">
-        <v>Model identifiers come from LG USA product URLs; this includes older/discontinued models.</v>
+        <v>Leave Count Qty A-B blank; zero is a recorded count of zero.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Source</v>
+        <v>Models</v>
       </c>
       <c r="B15" t="str">
-        <v>https://www.lg.com/us/sitemap.xml</v>
+        <v>Model identifiers come from LG USA product URLs; this includes older/discontinued models.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Source retrieved</v>
+        <v>Source</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-09-30</v>
+        <v>https://www.lg.com/us/sitemap.xml</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Distribution</v>
+        <v>Source retrieved</v>
       </c>
       <c r="B17" t="str">
-        <v>All 16 sections A-H, J-N, and P-R; P-R has sub-bays A-E.</v>
+        <v>2026-09-30</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
+        <v>Distribution</v>
+      </c>
+      <c r="B18" t="str">
+        <v>All 16 sections A-H, J-N, and P-R; P-R has sub-bays A-E.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
         <v>Persistence</v>
       </c>
-      <c r="B18" t="str">
+      <c r="B19" t="str">
         <v>Uploaded data lasts for this browser session only.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -33356,7 +33364,7 @@
         <v>Refrigerator</v>
       </c>
       <c r="C4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D4" t="str">
         <v>https://www.lg.com/us/refrigerators/lg-lcfs22exs-french-3-door-refrigerator</v>
@@ -33622,7 +33630,7 @@
         <v>Refrigerator</v>
       </c>
       <c r="C23">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D23" t="str">
         <v>https://www.lg.com/us/refrigerators/lg-LFXS29626W-french-3-door-refrigerator</v>
@@ -33818,7 +33826,7 @@
         <v>Refrigerator</v>
       </c>
       <c r="C37">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D37" t="str">
         <v>https://www.lg.com/us/refrigerators/lg-lrfvs3006d-french-3-door-refrigerator</v>
@@ -34378,7 +34386,7 @@
         <v>Washer</v>
       </c>
       <c r="C77">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D77" t="str">
         <v>https://www.lg.com/us/washers/lg-WM3700HWA-front-load-washer</v>
@@ -35456,7 +35464,7 @@
         <v>Dryer</v>
       </c>
       <c r="C154">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D154" t="str">
         <v>https://www.lg.com/us/dryers/lg-DLGX5681V-gas-dryer</v>
@@ -35974,7 +35982,7 @@
         <v>Dishwasher</v>
       </c>
       <c r="C191">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D191" t="str">
         <v>https://www.lg.com/us/dishwashers/lg-LDT5678ST-top-control-dishwasher</v>

</xml_diff>